<commit_message>
ci: update VSD data with embedded HTML (415 records) - 2026-06-15T11:06:10Z
</commit_message>
<xml_diff>
--- a/data/vsd_records.xlsx
+++ b/data/vsd_records.xlsx
@@ -602,7 +602,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:21</t>
+          <t>15/06/2026 17:52:34</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -736,7 +736,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:22</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -834,7 +834,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:22</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:22</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1030,7 +1030,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:22</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1155,7 +1155,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:22</t>
+          <t>15/06/2026 17:52:35</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1278,7 +1278,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:22</t>
+          <t>15/06/2026 17:52:35</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1408,7 +1408,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:22</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1506,7 +1506,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:22</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:22</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1798,7 +1798,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1944,7 +1944,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2090,7 +2090,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2236,7 +2236,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2382,7 +2382,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:36</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2674,7 +2674,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2820,7 +2820,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2966,7 +2966,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -3112,7 +3112,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -3258,7 +3258,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -3404,7 +3404,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -3550,7 +3550,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:23</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -3696,7 +3696,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -3842,7 +3842,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3988,7 +3988,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -4134,7 +4134,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -4280,7 +4280,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -4426,7 +4426,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:37</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -4718,7 +4718,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -4864,7 +4864,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -5010,7 +5010,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -5156,7 +5156,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -5302,7 +5302,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -5594,7 +5594,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:24</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -5740,7 +5740,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -5886,7 +5886,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -6032,7 +6032,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -6178,7 +6178,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -6324,7 +6324,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -6470,7 +6470,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -6616,7 +6616,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:38</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -6762,7 +6762,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -6908,7 +6908,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -7054,7 +7054,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -7200,7 +7200,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -7290,7 +7290,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:25</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -7436,7 +7436,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -7582,7 +7582,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -7728,7 +7728,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -7873,7 +7873,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -8006,7 +8006,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -8131,7 +8131,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -8277,7 +8277,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -8423,7 +8423,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:39</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -8569,7 +8569,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -8715,7 +8715,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -8848,7 +8848,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -8981,7 +8981,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -9107,7 +9107,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -9237,7 +9237,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -9367,7 +9367,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:26</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -9497,7 +9497,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -9627,7 +9627,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -9757,7 +9757,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -9880,7 +9880,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -10010,7 +10010,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -10154,7 +10154,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:40</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -10288,7 +10288,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -10385,7 +10385,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -10461,7 +10461,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -10537,7 +10537,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -10613,7 +10613,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -10711,7 +10711,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -10809,7 +10809,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -10899,7 +10899,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:27</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -11038,7 +11038,7 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
@@ -11172,7 +11172,7 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
@@ -11306,7 +11306,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -11441,7 +11441,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -11576,7 +11576,7 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
@@ -11699,7 +11699,7 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
@@ -11822,7 +11822,7 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:41</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -11952,7 +11952,7 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -12075,7 +12075,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -12125,7 +12125,11 @@
 CTCP tập đoàn cơ khí Công nghệ cao Siba và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="E88" t="inlineStr"/>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>SBG</t>
+        </is>
+      </c>
       <c r="F88" t="inlineStr">
         <is>
           <t>Thực hiện quyền nhận cổ tức bằng cổ phiếu</t>
@@ -12146,11 +12150,7 @@
           <t>VN000000SBG1</t>
         </is>
       </c>
-      <c r="J88" t="inlineStr">
-        <is>
-          <t>SBG</t>
-        </is>
-      </c>
+      <c r="J88" t="inlineStr"/>
       <c r="K88" t="inlineStr">
         <is>
           <t>26/06/2026</t>
@@ -12163,7 +12163,11 @@
       </c>
       <c r="M88" t="inlineStr"/>
       <c r="N88" t="inlineStr"/>
-      <c r="O88" t="inlineStr"/>
+      <c r="O88" t="inlineStr">
+        <is>
+          <t>31/07/2026</t>
+        </is>
+      </c>
       <c r="P88" t="inlineStr"/>
       <c r="Q88" t="inlineStr"/>
       <c r="R88" t="inlineStr"/>
@@ -12178,7 +12182,7 @@
       <c r="W88" t="inlineStr"/>
       <c r="X88" t="inlineStr">
         <is>
-          <t>Thực hiện quyền nhận cổ tức bằng cổ phiếu - a. Thực hiện quyền nhận cổ tức bằng cổ phiếu - Tỷ lệ thực hiện: 100:20 (Mỗi cổ đông nắm giữ 100 cổ phiếu sẽ được nhận thêm 20 cổ phiếu mới) - Phương án làm tròn, phương án xử lý cổ phiếu lẻ (nếu có): Số lượng cổ phiếu phát hành thêm cho cổ đông hiện hữu sẽ được làm tròn xuống đến hàng đơn vị, phần cổ phiếu lẻ phát sinh (nếu có) sẽ bị hủy bỏ. - Ví dụ: Tại ngày chốt danh sách cổ đông để thực hiện quyền, cổ đông A sở hữu 2.026 cổ phiếu SBG. Cổ đông A sẽ nhận được thêm: (2.026/100)*20= 405,2 cổ phiếu SBG. Theo nguyên tắc làm tròn, cổ đông A nhận được 405 cổ phiếu SBG, phần lẻ là 0,2 cổ phiếu sẽ bị hủy bỏ - Địa điểm thực hiện: + Đối với chứng khoán lưu ký: Người sở hữu chứng khoán nhận cổ tức bằng cổ phiếu tại các thành viên lưu ký nơi mở tài khoản lưu ký, tổ chức mở tài khoản trực tiếp tại VSDC. + Đối với chứng khoán chưa lưu ký: Người sở hữu chứng khoán làm thủ tục nhận cổ tức bằng cổ phiếu tại văn phòng đại diện của Công ty Cổ phần Tập đoàn Cơ khí Công nghệ cao Siba - Tầng 7, Tòa nhà Vista Tower, 628C đường Võ Nguyên Giáp, Phường An Khánh, Thành phố Hồ Chí Minh và xuất trình căn cước công dân/căn cước.</t>
+          <t>Thực hiện quyền nhận cổ tức bằng cổ phiếu - Tỷ lệ thực hiện: 100:20 (Mỗi cổ đông nắm giữ 100 cổ phiếu sẽ được nhận thêm 20 cổ phiếu mới) - Thời gian thực hiện: Dự kiến trong tháng 7/2026. Thời gian cụ thể sẽ thông báo đến cổ đông trong Phiếu lấy ý kiến cổ đông bằng văn bản.</t>
         </is>
       </c>
       <c r="Y88" t="n">
@@ -12209,7 +12213,7 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -12259,7 +12263,11 @@
 CTCP tập đoàn cơ khí Công nghệ cao Siba và các tổ chức, cá nhân tham gia vào quá trình lập hồ sơ, tài liệu thực hiện quyền phải chịu trách nhiệm trước pháp luật về tính hợp pháp, chính xác, trung thực và đầy đủ của hồ sơ; Tổ chức, cá nhân tham gia vào xác nhận hồ sơ, tài liệu phải chịu trách nhiệm trước pháp luật trong phạm vi liên quan đến hồ sơ, tài liệu đó theo quy định tại khoản 1 Điều 11a Luật Chứng khoán số 54/2019/QH14 ngày 26/11/2019 được bổ sung tại khoản 4 Điều 1 Luật số 56/2024/QH15 ngày 29/11/2024./.</t>
         </is>
       </c>
-      <c r="E89" t="inlineStr"/>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>SBG</t>
+        </is>
+      </c>
       <c r="F89" t="inlineStr">
         <is>
           <t>Thực hiện lấy ý kiến cổ đông bằng văn bản lần 1 năm 2026</t>
@@ -12276,11 +12284,7 @@
           <t>VN000000SBG1</t>
         </is>
       </c>
-      <c r="J89" t="inlineStr">
-        <is>
-          <t>SBG</t>
-        </is>
-      </c>
+      <c r="J89" t="inlineStr"/>
       <c r="K89" t="inlineStr">
         <is>
           <t>26/06/2026</t>
@@ -12343,7 +12347,7 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -12477,7 +12481,7 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:28</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -12613,7 +12617,7 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -12738,7 +12742,7 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -12872,7 +12876,7 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
@@ -13021,7 +13025,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
@@ -13170,7 +13174,7 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
@@ -13311,7 +13315,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -13452,7 +13456,7 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:42</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
@@ -13593,7 +13597,7 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
@@ -13734,7 +13738,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -13869,7 +13873,7 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
@@ -14038,7 +14042,7 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
@@ -14161,7 +14165,7 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
@@ -14286,7 +14290,7 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
@@ -14426,7 +14430,7 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
@@ -14564,7 +14568,7 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -14703,7 +14707,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
@@ -14822,7 +14826,7 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:29</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
@@ -14956,7 +14960,7 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
@@ -15086,7 +15090,7 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
@@ -15221,7 +15225,7 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
@@ -15319,7 +15323,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
@@ -15417,7 +15421,7 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -15515,7 +15519,7 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:43</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -15613,7 +15617,7 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -15738,7 +15742,7 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -15836,7 +15840,7 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -15933,7 +15937,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -16031,7 +16035,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -16161,7 +16165,7 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:30</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -16295,7 +16299,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
@@ -16425,7 +16429,7 @@
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
@@ -16555,7 +16559,7 @@
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
@@ -16689,7 +16693,7 @@
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
@@ -16835,7 +16839,7 @@
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
@@ -16981,7 +16985,7 @@
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:44</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
@@ -17127,7 +17131,7 @@
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
@@ -17273,7 +17277,7 @@
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
@@ -17419,7 +17423,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
@@ -17565,7 +17569,7 @@
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
@@ -17711,7 +17715,7 @@
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -17857,7 +17861,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
@@ -18003,7 +18007,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:31</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
@@ -18149,7 +18153,7 @@
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
@@ -18295,7 +18299,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
@@ -18441,7 +18445,7 @@
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -18587,7 +18591,7 @@
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
@@ -18691,7 +18695,7 @@
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
@@ -18795,7 +18799,7 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
@@ -18872,7 +18876,7 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:45</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
@@ -19011,7 +19015,7 @@
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
@@ -19150,7 +19154,7 @@
       </c>
       <c r="B142" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C142" t="inlineStr">
@@ -19289,7 +19293,7 @@
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -19428,7 +19432,7 @@
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -19567,7 +19571,7 @@
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -19705,7 +19709,7 @@
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -19835,7 +19839,7 @@
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
@@ -19965,7 +19969,7 @@
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:32</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
@@ -20095,7 +20099,7 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
@@ -20225,7 +20229,7 @@
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
@@ -20355,7 +20359,7 @@
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
@@ -20453,7 +20457,7 @@
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
@@ -20588,7 +20592,7 @@
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:46</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
@@ -20714,7 +20718,7 @@
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
@@ -20842,7 +20846,7 @@
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -20971,7 +20975,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -21101,7 +21105,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -21231,7 +21235,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -21360,7 +21364,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -21490,7 +21494,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -21620,7 +21624,7 @@
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:33</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -21750,7 +21754,7 @@
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -21879,7 +21883,7 @@
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -22008,7 +22012,7 @@
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
@@ -22137,7 +22141,7 @@
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -22271,7 +22275,7 @@
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:47</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -22398,7 +22402,7 @@
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
@@ -22525,7 +22529,7 @@
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
@@ -22655,7 +22659,7 @@
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -22780,7 +22784,7 @@
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -22910,7 +22914,7 @@
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
@@ -22979,7 +22983,7 @@
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
@@ -23090,7 +23094,7 @@
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:34</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
@@ -23170,7 +23174,7 @@
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
@@ -23278,7 +23282,7 @@
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
@@ -23417,7 +23421,7 @@
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -23532,7 +23536,7 @@
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -23647,7 +23651,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -23750,7 +23754,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -23853,7 +23857,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:48</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -23956,7 +23960,7 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
@@ -24059,7 +24063,7 @@
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -24185,7 +24189,7 @@
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -24320,7 +24324,7 @@
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
@@ -24418,7 +24422,7 @@
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
@@ -24550,7 +24554,7 @@
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:35</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -24675,7 +24679,7 @@
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
@@ -24805,7 +24809,7 @@
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
@@ -24935,7 +24939,7 @@
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
@@ -25065,7 +25069,7 @@
       </c>
       <c r="B190" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C190" t="inlineStr">
@@ -25207,7 +25211,7 @@
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
@@ -25349,7 +25353,7 @@
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
@@ -25482,7 +25486,7 @@
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -25616,7 +25620,7 @@
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:49</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -25750,7 +25754,7 @@
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -25876,7 +25880,7 @@
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -26010,7 +26014,7 @@
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -26135,7 +26139,7 @@
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -26269,7 +26273,7 @@
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
@@ -26408,7 +26412,7 @@
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
@@ -26547,7 +26551,7 @@
       </c>
       <c r="B201" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C201" t="inlineStr">
@@ -26636,7 +26640,7 @@
       </c>
       <c r="B202" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:36</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C202" t="inlineStr">
@@ -26726,7 +26730,7 @@
       </c>
       <c r="B203" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:37</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C203" t="inlineStr">
@@ -26864,7 +26868,7 @@
       </c>
       <c r="B204" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:37</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C204" t="inlineStr">
@@ -27003,7 +27007,7 @@
       </c>
       <c r="B205" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:37</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C205" t="inlineStr">
@@ -27142,7 +27146,7 @@
       </c>
       <c r="B206" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:37</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C206" t="inlineStr">
@@ -27272,7 +27276,7 @@
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:37</t>
+          <t>15/06/2026 17:52:50</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
@@ -27406,7 +27410,7 @@
       </c>
       <c r="B208" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:37</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C208" t="inlineStr">
@@ -27540,7 +27544,7 @@
       </c>
       <c r="B209" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:37</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C209" t="inlineStr">
@@ -27679,7 +27683,7 @@
       </c>
       <c r="B210" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:37</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C210" t="inlineStr">
@@ -27784,7 +27788,7 @@
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -27882,7 +27886,7 @@
       </c>
       <c r="B212" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:37</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C212" t="inlineStr">
@@ -27980,7 +27984,7 @@
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -28103,7 +28107,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -28233,7 +28237,7 @@
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -28363,7 +28367,7 @@
       </c>
       <c r="B216" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C216" t="inlineStr">
@@ -28486,7 +28490,7 @@
       </c>
       <c r="B217" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C217" t="inlineStr">
@@ -28616,7 +28620,7 @@
       </c>
       <c r="B218" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C218" t="inlineStr">
@@ -28739,7 +28743,7 @@
       </c>
       <c r="B219" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C219" t="inlineStr">
@@ -28869,7 +28873,7 @@
       </c>
       <c r="B220" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:51</t>
         </is>
       </c>
       <c r="C220" t="inlineStr">
@@ -28999,7 +29003,7 @@
       </c>
       <c r="B221" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C221" t="inlineStr">
@@ -29129,7 +29133,7 @@
       </c>
       <c r="B222" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C222" t="inlineStr">
@@ -29260,7 +29264,7 @@
       </c>
       <c r="B223" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C223" t="inlineStr">
@@ -29394,7 +29398,7 @@
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
@@ -29528,7 +29532,7 @@
       </c>
       <c r="B225" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C225" t="inlineStr">
@@ -29662,7 +29666,7 @@
       </c>
       <c r="B226" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:38</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C226" t="inlineStr">
@@ -29798,7 +29802,7 @@
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:39</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
@@ -29934,7 +29938,7 @@
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:39</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -30070,7 +30074,7 @@
       </c>
       <c r="B229" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:39</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C229" t="inlineStr">
@@ -30205,7 +30209,7 @@
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:39</t>
+          <t>15/06/2026 17:52:53</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -30339,7 +30343,7 @@
       </c>
       <c r="B231" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:39</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C231" t="inlineStr">
@@ -30473,7 +30477,7 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:39</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
@@ -30602,7 +30606,7 @@
       </c>
       <c r="B233" t="inlineStr">
         <is>
-          <t>15/06/2026 16:55:39</t>
+          <t>15/06/2026 17:52:52</t>
         </is>
       </c>
       <c r="C233" t="inlineStr">

</xml_diff>